<commit_message>
chore(weekly-sync): auto-pull through 2026-08-23
</commit_message>
<xml_diff>
--- a/data/raw/returns/Audio Array.xlsx
+++ b/data/raw/returns/Audio Array.xlsx
@@ -3554,27 +3554,27 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>406-6095938-9247562</t>
+          <t>406-4803906-5357102</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>FBA75674</t>
+          <t>FBA79840</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>B0B4G19R58</t>
+          <t>B0FQBWV1ST</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>X001L4QVU5</t>
+          <t>X002EDSRBN</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Audio Array Mic | Podcast Mic XLR Condenser Microphone Kit with Boom Arm | Pop Filter | Shock Mount &amp; 2M Cable | Cardioid Recording Microphone for Streaming | Podcasting &amp; Home Studio | AM-C2</t>
+          <t>Audio Array AH-60-RD Semi-Open Back DJ Headphones | 50mm Drivers Delivers Dynamic Balanced Output | 15Hz-25kHz, 32Ω, 100dB SPL, 1200mW | 3m OFC Single-Sided Cable with Screw-On 3.5mm + 6.3mm Plug</t>
         </is>
       </c>
       <c r="G56" t="n">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>LPNDEL5S14658333</t>
+          <t>LPNDEL5S14658334</t>
         </is>
       </c>
       <c r="L56" t="inlineStr"/>
@@ -3610,27 +3610,27 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>406-4803906-5357102</t>
+          <t>406-6095938-9247562</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>FBA79840</t>
+          <t>FBA75674</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>B0FQBWV1ST</t>
+          <t>B0B4G19R58</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>X002EDSRBN</t>
+          <t>X001L4QVU5</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Audio Array AH-60-RD Semi-Open Back DJ Headphones | 50mm Drivers Delivers Dynamic Balanced Output | 15Hz-25kHz, 32Ω, 100dB SPL, 1200mW | 3m OFC Single-Sided Cable with Screw-On 3.5mm + 6.3mm Plug</t>
+          <t>Audio Array Mic | Podcast Mic XLR Condenser Microphone Kit with Boom Arm | Pop Filter | Shock Mount &amp; 2M Cable | Cardioid Recording Microphone for Streaming | Podcasting &amp; Home Studio | AM-C2</t>
         </is>
       </c>
       <c r="G57" t="n">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>LPNDEL5S14658334</t>
+          <t>LPNDEL5S14658333</t>
         </is>
       </c>
       <c r="L57" t="inlineStr"/>
@@ -30934,7 +30934,7 @@
       </c>
       <c r="B540" t="inlineStr">
         <is>
-          <t>405-9316299-5823523</t>
+          <t>405-3372664-3710705</t>
         </is>
       </c>
       <c r="C540" t="inlineStr">
@@ -30977,7 +30977,7 @@
       </c>
       <c r="K540" t="inlineStr">
         <is>
-          <t>LPNCJB1X148070</t>
+          <t>LPNCJB1X148074</t>
         </is>
       </c>
       <c r="L540" t="inlineStr"/>
@@ -30990,7 +30990,7 @@
       </c>
       <c r="B541" t="inlineStr">
         <is>
-          <t>405-3372664-3710705</t>
+          <t>405-9316299-5823523</t>
         </is>
       </c>
       <c r="C541" t="inlineStr">
@@ -31033,7 +31033,7 @@
       </c>
       <c r="K541" t="inlineStr">
         <is>
-          <t>LPNCJB1X148074</t>
+          <t>LPNCJB1X148070</t>
         </is>
       </c>
       <c r="L541" t="inlineStr"/>

</xml_diff>